<commit_message>
feat(link-remodeling): Fix Excel import for links
</commit_message>
<xml_diff>
--- a/TurboVault TPCH Data.xlsx
+++ b/TurboVault TPCH Data.xlsx
@@ -3,17 +3,17 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="source_data" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="standard_hub" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="standard_link" sheetId="3" r:id="rId6"/>
-    <sheet state="visible" name="standard_satellite" sheetId="4" r:id="rId7"/>
-    <sheet state="visible" name="multiactive_satellite" sheetId="5" r:id="rId8"/>
-    <sheet state="visible" name="non_historized_link" sheetId="6" r:id="rId9"/>
-    <sheet state="visible" name="non_historized_satellite" sheetId="7" r:id="rId10"/>
-    <sheet state="visible" name="ref_table" sheetId="8" r:id="rId11"/>
-    <sheet state="visible" name="ref_hub" sheetId="9" r:id="rId12"/>
-    <sheet state="visible" name="ref_sat" sheetId="10" r:id="rId13"/>
-    <sheet state="visible" name="pit" sheetId="11" r:id="rId14"/>
+    <sheet state="visible" name="source_data" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="standard_hub" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="standard_link" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="standard_satellite" sheetId="4" r:id="rId8"/>
+    <sheet state="visible" name="multiactive_satellite" sheetId="5" r:id="rId9"/>
+    <sheet state="visible" name="non_historized_link" sheetId="6" r:id="rId10"/>
+    <sheet state="visible" name="non_historized_satellite" sheetId="7" r:id="rId11"/>
+    <sheet state="visible" name="ref_table" sheetId="8" r:id="rId12"/>
+    <sheet state="visible" name="ref_hub" sheetId="9" r:id="rId13"/>
+    <sheet state="visible" name="ref_sat" sheetId="10" r:id="rId14"/>
+    <sheet state="visible" name="pit" sheetId="11" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="260">
   <si>
     <t>Source_table_identifier</t>
   </si>
@@ -192,9 +192,6 @@
     <t>hub with 1 bk and 2 sources</t>
   </si>
   <si>
-    <t>SRC004</t>
-  </si>
-  <si>
     <t>C_CustomerKey</t>
   </si>
   <si>
@@ -339,24 +336,33 @@
     <t>HK_ORDERS_CUSTOMERS_L</t>
   </si>
   <si>
+    <t>1 src, 2 hubs with 1 bk each + dependant child key</t>
+  </si>
+  <si>
+    <t>O_CUSTKEY</t>
+  </si>
+  <si>
+    <t>O_COMMENT</t>
+  </si>
+  <si>
+    <t>DCK_COMMENT</t>
+  </si>
+  <si>
+    <t>L0002</t>
+  </si>
+  <si>
+    <t>PART_SUPPLIER_L</t>
+  </si>
+  <si>
+    <t>PS_PARTKEY</t>
+  </si>
+  <si>
+    <t>HK_PART_SUPPLIER_L</t>
+  </si>
+  <si>
     <t>1 src, 2 hubs with 1 bk each</t>
   </si>
   <si>
-    <t>O_CUSTKEY</t>
-  </si>
-  <si>
-    <t>L0002</t>
-  </si>
-  <si>
-    <t>PART_SUPPLIER_L</t>
-  </si>
-  <si>
-    <t>PS_PARTKEY</t>
-  </si>
-  <si>
-    <t>HK_PART_SUPPLIER_L</t>
-  </si>
-  <si>
     <t>PS_SUPPKEY</t>
   </si>
   <si>
@@ -384,6 +390,21 @@
     <t>1 src, 2 hubs, prejoin and 2bk components</t>
   </si>
   <si>
+    <t>L0005</t>
+  </si>
+  <si>
+    <t>customer_duplicate_customer_l</t>
+  </si>
+  <si>
+    <t>hk_customer_duplicate_customer_l</t>
+  </si>
+  <si>
+    <t>link pointing to the same hub twice</t>
+  </si>
+  <si>
+    <t>HK_CUSTOMER_DUPLICATE_H</t>
+  </si>
+  <si>
     <t>Satellite_Identifier</t>
   </si>
   <si>
@@ -436,9 +457,6 @@
   </si>
   <si>
     <t>O_CLERK</t>
-  </si>
-  <si>
-    <t>O_COMMENT</t>
   </si>
   <si>
     <t>O_ORDERDATE</t>
@@ -953,6 +971,10 @@
 
 <file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2441,16 +2463,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="15" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="C1" s="15" t="s">
         <v>39</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="E1" s="15" t="s">
         <v>40</v>
@@ -2463,19 +2485,19 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="F2" s="6">
         <v>1.0</v>
@@ -2483,19 +2505,19 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="F3" s="6">
         <v>2.0</v>
@@ -2503,19 +2525,19 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="F4" s="6">
         <v>3.0</v>
@@ -2523,19 +2545,19 @@
     </row>
     <row r="5">
       <c r="A5" s="6" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="F5" s="6">
         <v>1.0</v>
@@ -2543,19 +2565,19 @@
     </row>
     <row r="6">
       <c r="A6" s="6" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="F6" s="6">
         <v>2.0</v>
@@ -2563,19 +2585,19 @@
     </row>
     <row r="7">
       <c r="A7" s="6" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="F7" s="6">
         <v>3.0</v>
@@ -2607,25 +2629,25 @@
   <sheetData>
     <row r="1" ht="39.0" customHeight="1">
       <c r="A1" s="7" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="H1" s="7" t="s">
         <v>8</v>
@@ -2633,25 +2655,25 @@
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>49</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="H2" s="6" t="s">
         <v>52</v>
@@ -3765,10 +3787,10 @@
         <v>49</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>54</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>55</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>50</v>
@@ -3795,25 +3817,25 @@
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>56</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>57</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F4" s="3">
         <v>1.0</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H4" s="6">
         <v>0.0</v>
@@ -3828,25 +3850,25 @@
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>60</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>61</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F5" s="3">
         <v>1.0</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H5" s="6">
         <v>0.0</v>
@@ -3855,31 +3877,31 @@
         <v>1.0</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K5" s="9"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>65</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>66</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F6" s="3">
         <v>1.0</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H6" s="6">
         <v>0.0</v>
@@ -3888,30 +3910,30 @@
         <v>1.0</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>70</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>71</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D7" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>72</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>73</v>
       </c>
       <c r="F7" s="6">
         <v>1.0</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H7" s="6">
         <v>0.0</v>
@@ -3923,30 +3945,30 @@
         <v>32</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>70</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>71</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D8" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>77</v>
       </c>
       <c r="F8" s="6">
         <v>2.0</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H8" s="6">
         <v>0.0</v>
@@ -3958,30 +3980,30 @@
         <v>32</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>78</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>79</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D9" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>72</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>73</v>
       </c>
       <c r="F9" s="6">
         <v>1.0</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H9" s="6">
         <v>0.0</v>
@@ -3993,30 +4015,30 @@
         <v>32</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>78</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>79</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D10" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>77</v>
       </c>
       <c r="F10" s="6">
         <v>2.0</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H10" s="6">
         <v>0.0</v>
@@ -4028,30 +4050,30 @@
         <v>32</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>78</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>79</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F11" s="6">
         <v>1.0</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H11" s="6">
         <v>0.0</v>
@@ -4063,30 +4085,30 @@
         <v>32</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>78</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>79</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F12" s="6">
         <v>2.0</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H12" s="6">
         <v>0.0</v>
@@ -4098,30 +4120,30 @@
         <v>32</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>82</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>83</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D13" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="E13" s="6" t="s">
         <v>84</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>85</v>
       </c>
       <c r="F13" s="6">
         <v>1.0</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H13" s="6">
         <v>0.0</v>
@@ -4135,25 +4157,25 @@
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>87</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>88</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F14" s="6">
         <v>1.0</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H14" s="6">
         <v>0.0</v>
@@ -5185,37 +5207,37 @@
   <sheetData>
     <row r="1" ht="48.0" customHeight="1">
       <c r="A1" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>90</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>91</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>39</v>
       </c>
       <c r="D1" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="F1" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="G1" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="H1" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="I1" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="J1" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="K1" s="10" t="s">
         <v>98</v>
-      </c>
-      <c r="K1" s="10" t="s">
-        <v>99</v>
       </c>
       <c r="L1" s="10" t="s">
         <v>42</v>
@@ -5235,31 +5257,31 @@
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>100</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>101</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="J2" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>59</v>
-      </c>
       <c r="K2" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="L2" s="3">
         <v>1.0</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N2" s="6">
         <v>0.0</v>
@@ -5268,21 +5290,21 @@
         <v>17</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>100</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>101</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>48</v>
@@ -5297,7 +5319,7 @@
         <v>2.0</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N3" s="6">
         <v>0.0</v>
@@ -5306,162 +5328,154 @@
         <v>17</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>63</v>
-      </c>
       <c r="L4" s="3">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="N4" s="6">
-        <v>0.0</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>64</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
       <c r="P4" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="C5" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>28</v>
       </c>
       <c r="D5" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="L5" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="M5" s="3" t="s">
         <v>109</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="L5" s="3">
-        <v>2.0</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>108</v>
       </c>
       <c r="N5" s="6">
         <v>0.0</v>
       </c>
       <c r="O5" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="I6" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="P5" s="6" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="L6" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="M6" s="6" t="s">
-        <v>112</v>
+      <c r="J6" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="L6" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>109</v>
       </c>
       <c r="N6" s="6">
         <v>0.0</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>35</v>
+        <v>63</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>72</v>
+        <v>75</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>84</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="K7" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="L7" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="M7" s="6" t="s">
         <v>114</v>
-      </c>
-      <c r="L7" s="6">
-        <v>2.0</v>
-      </c>
-      <c r="M7" s="6" t="s">
-        <v>112</v>
       </c>
       <c r="N7" s="6">
         <v>0.0</v>
@@ -5470,48 +5484,36 @@
         <v>35</v>
       </c>
       <c r="P7" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="6" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>86</v>
+        <v>116</v>
       </c>
       <c r="L8" s="6">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="N8" s="6">
         <v>0.0</v>
@@ -5520,36 +5522,48 @@
         <v>35</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>72</v>
+        <v>75</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>84</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="L9" s="6">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="N9" s="6">
         <v>0.0</v>
@@ -5558,36 +5572,36 @@
         <v>35</v>
       </c>
       <c r="P9" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L10" s="6">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="M10" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="N10" s="6">
         <v>0.0</v>
@@ -5596,12 +5610,123 @@
         <v>35</v>
       </c>
       <c r="P10" s="6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" ht="15.75" customHeight="1">
+      <c r="A11" s="6" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="11" ht="15.75" customHeight="1"/>
-    <row r="12" ht="15.75" customHeight="1"/>
-    <row r="13" ht="15.75" customHeight="1"/>
+      <c r="B11" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="L11" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="M11" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="N11" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="O11" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="P11" s="6" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="L12" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="M12" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="N12" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="O12" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="P12" s="6" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="L13" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="M13" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="N13" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="O13" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="P13" s="6" t="s">
+        <v>123</v>
+      </c>
+    </row>
     <row r="14" ht="15.75" customHeight="1"/>
     <row r="15" ht="15.75" customHeight="1"/>
     <row r="16" ht="15.75" customHeight="1"/>
@@ -6587,6 +6712,7 @@
     <row r="996" ht="15.75" customHeight="1"/>
     <row r="997" ht="15.75" customHeight="1"/>
     <row r="998" ht="15.75" customHeight="1"/>
+    <row r="999" ht="15.75" customHeight="1"/>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
@@ -6616,10 +6742,10 @@
   <sheetData>
     <row r="1" ht="48.0" customHeight="1">
       <c r="A1" s="7" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>39</v>
@@ -6628,13 +6754,13 @@
         <v>40</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="H1" s="7" t="s">
         <v>42</v>
@@ -6645,26 +6771,26 @@
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>48</v>
       </c>
       <c r="F2" s="2" t="str">
-        <f>VLOOKUP(E2, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(E2, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_CUSTOMER_H</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="H2" s="2">
         <v>1.0</v>
@@ -6675,26 +6801,26 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>48</v>
       </c>
       <c r="F3" s="2" t="str">
-        <f>VLOOKUP(E3, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(E3, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_CUSTOMER_H</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="H3" s="2">
         <v>2.0</v>
@@ -6705,26 +6831,26 @@
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>48</v>
       </c>
       <c r="F4" s="2" t="str">
-        <f>VLOOKUP(E4, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(E4, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_CUSTOMER_H</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="H4" s="2">
         <v>3.0</v>
@@ -6735,26 +6861,26 @@
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>48</v>
       </c>
       <c r="F5" s="2" t="str">
-        <f>VLOOKUP(E5, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(E5, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_CUSTOMER_H</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="H5" s="2">
         <v>1.0</v>
@@ -6765,26 +6891,26 @@
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>48</v>
       </c>
       <c r="F6" s="2" t="str">
-        <f>VLOOKUP(E6, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(E6, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_CUSTOMER_H</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="H6" s="2">
         <v>2.0</v>
@@ -6795,26 +6921,26 @@
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="3" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>48</v>
       </c>
       <c r="F7" s="2" t="str">
-        <f>VLOOKUP(E7, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(E7, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_CUSTOMER_H</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="H7" s="2">
         <v>3.0</v>
@@ -6825,26 +6951,26 @@
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F8" s="3" t="str">
-        <f>VLOOKUP(E8, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(E8, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_ORDER_H</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="H8" s="3">
         <v>1.0</v>
@@ -6855,26 +6981,26 @@
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>136</v>
+        <v>104</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F9" s="3" t="str">
-        <f>VLOOKUP(E9, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(E9, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_ORDER_H</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>136</v>
+        <v>104</v>
       </c>
       <c r="H9" s="3">
         <v>2.0</v>
@@ -6885,26 +7011,26 @@
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F10" s="3" t="str">
-        <f>VLOOKUP(E10, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(E10, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_ORDER_H</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="H10" s="3">
         <v>3.0</v>
@@ -6915,26 +7041,26 @@
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F11" s="3" t="str">
-        <f>VLOOKUP(E11, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(E11, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_ORDER_H</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="H11" s="3">
         <v>4.0</v>
@@ -6945,26 +7071,26 @@
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="3" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F12" s="3" t="str">
-        <f>VLOOKUP(E12, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(E12, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_ORDER_H</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="H12" s="3">
         <v>5.0</v>
@@ -6975,26 +7101,26 @@
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="3" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F13" s="3" t="str">
-        <f>VLOOKUP(E13, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(E13, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_ORDER_H</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="H13" s="3">
         <v>6.0</v>
@@ -7005,26 +7131,26 @@
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="3" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F14" s="3" t="str">
-        <f>VLOOKUP(E14, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(E14, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_ORDER_H</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="H14" s="3">
         <v>7.0</v>
@@ -7035,382 +7161,382 @@
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="3" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F15" s="2" t="str">
-        <f>VLOOKUP(E15, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(E15, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_SUPPLIER_H</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="H15" s="3">
         <v>1.0</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="3" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F16" s="2" t="str">
-        <f>VLOOKUP(E16, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(E16, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_SUPPLIER_H</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="H16" s="3">
         <v>2.0</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="3" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>25</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F17" s="2" t="str">
-        <f>VLOOKUP(E17, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(E17, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_SUPPLIER_H</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="H17" s="3">
         <v>1.0</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="3" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>28</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="H18" s="3">
         <v>1.0</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="3" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>28</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="H19" s="3">
         <v>2.0</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="3" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>28</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="H20" s="3">
         <v>3.0</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="3" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="H21" s="3">
         <v>1.0</v>
       </c>
       <c r="I21" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="3" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="H22" s="3">
         <v>2.0</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="3" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="H23" s="3">
         <v>3.0</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="3" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="H24" s="3">
         <v>4.0</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="3" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="H25" s="6">
         <v>5.0</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="3" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="H26" s="6">
         <v>6.0</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="3" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="H27" s="6">
         <v>7.0</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>
@@ -8416,28 +8542,28 @@
   <sheetData>
     <row r="1" ht="48.0" customHeight="1">
       <c r="A1" s="10" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I1" s="7" t="s">
         <v>42</v>
@@ -8446,21 +8572,21 @@
         <v>8</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>48</v>
@@ -8469,10 +8595,10 @@
         <v>49</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="I2" s="3">
         <v>1.0</v>
@@ -8481,21 +8607,21 @@
         <v>11</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>48</v>
@@ -8504,10 +8630,10 @@
         <v>49</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="I3" s="3">
         <v>2.0</v>
@@ -8518,16 +8644,16 @@
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>48</v>
@@ -8536,7 +8662,7 @@
         <v>49</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="H4" s="3"/>
       <c r="I4" s="3">
@@ -8546,33 +8672,33 @@
         <v>11</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>61</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="I5" s="3">
         <v>1.0</v>
@@ -8581,30 +8707,30 @@
         <v>20</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>19</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="E6" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>61</v>
-      </c>
       <c r="G6" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="H6" s="3"/>
       <c r="I6" s="3">
@@ -8614,7 +8740,7 @@
         <v>20</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
@@ -9669,37 +9795,37 @@
   <sheetData>
     <row r="1" ht="48.0" customHeight="1">
       <c r="A1" s="10" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>39</v>
       </c>
       <c r="D1" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="F1" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="G1" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="H1" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="I1" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="J1" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="K1" s="10" t="s">
         <v>98</v>
-      </c>
-      <c r="K1" s="10" t="s">
-        <v>99</v>
       </c>
       <c r="L1" s="10" t="s">
         <v>42</v>
@@ -9716,32 +9842,32 @@
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J2" s="3" t="str">
-        <f>VLOOKUP(I2, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(I2, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_PART_H</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L2" s="3">
         <v>1.0</v>
       </c>
       <c r="M2" s="13" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="N2" s="6">
         <v>0.0</v>
@@ -9752,32 +9878,32 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="J3" s="3" t="str">
-        <f>VLOOKUP(I3, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(I3, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_ORDER_H</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="L3" s="3">
         <v>2.0</v>
       </c>
       <c r="M3" s="13" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="N3" s="6">
         <v>0.0</v>
@@ -9788,32 +9914,32 @@
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J4" s="8" t="str">
-        <f>VLOOKUP(I4, standard_link!$I$1:$O$5, 2, FALSE)</f>
+        <f>VLOOKUP(I4, standard_link!$I$1:$O$6, 2, FALSE)</f>
         <v>HK_SUPPLIER_H</v>
       </c>
       <c r="K4" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="L4" s="6">
         <v>3.0</v>
       </c>
       <c r="M4" s="13" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="N4" s="6">
         <v>0.0</v>
@@ -9824,25 +9950,25 @@
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="L5" s="3">
         <v>4.0</v>
       </c>
       <c r="M5" s="13" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="N5" s="6">
         <v>0.0</v>
@@ -9853,19 +9979,19 @@
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="L6" s="3">
         <v>5.0</v>
@@ -9880,19 +10006,19 @@
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="L7" s="6">
         <v>6.0</v>
@@ -9907,19 +10033,19 @@
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="L8" s="3">
         <v>7.0</v>
@@ -9934,19 +10060,19 @@
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="L9" s="3">
         <v>8.0</v>
@@ -9961,19 +10087,19 @@
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="L10" s="6">
         <v>9.0</v>
@@ -9988,19 +10114,19 @@
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="L11" s="3">
         <v>10.0</v>
@@ -10015,19 +10141,19 @@
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="L12" s="3">
         <v>11.0</v>
@@ -10042,19 +10168,19 @@
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="L13" s="6">
         <v>12.0</v>
@@ -10069,19 +10195,19 @@
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="L14" s="3">
         <v>13.0</v>
@@ -10096,19 +10222,19 @@
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="L15" s="3">
         <v>14.0</v>
@@ -10123,19 +10249,19 @@
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="L16" s="3">
         <v>15.0</v>
@@ -10150,19 +10276,19 @@
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="L17" s="3">
         <v>16.0</v>
@@ -11197,10 +11323,10 @@
   <sheetData>
     <row r="1" ht="42.75" customHeight="1">
       <c r="A1" s="7" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>39</v>
@@ -11209,13 +11335,13 @@
         <v>40</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="H1" s="7" t="s">
         <v>8</v>
@@ -11223,80 +11349,80 @@
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -12415,25 +12541,25 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="15" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="H1" s="7" t="s">
         <v>8</v>
@@ -12441,48 +12567,48 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -12505,10 +12631,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="15" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="C1" s="15" t="s">
         <v>39</v>
@@ -12520,69 +12646,69 @@
         <v>42</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="G1" s="15"/>
       <c r="H1" s="7"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="E2" s="6">
         <v>1.0</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="E3" s="6">
         <v>1.0</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="E4" s="6">
         <v>2.0</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>